<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.002-02 Le cerf-volant de papier
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.002-02.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.002-02.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>terrasse, lavande, après la sieste</t>
+          <t>terrasse, lavande, après la sieste, pierre chaude, tiges violettes</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Mila veut que son cerf-volant de papier se lève au-dessus de la lavande. Elle propose. Aniss dit je regarde, puis plus tard, puis non pour la ficelle. Mila accepte. Une abeille passe. L'ombre du cerf-volant glisse sur les fleurs.</t>
+          <t>La pierre de la terrasse tient la chaleur. Sur la pierre, un éclat de pierre brille. Mila veut le cerf-volant au-dessus des tiges, maintenant. Elle lève trop vite : le papier tombe. Sourire parti. Elle tend la ficelle à Aniss : il retire les doigts, il regarde. Elle refuse de foncer, attend, dit d'accord. Merci vécu. Elle tire d'un coup : le papier plonge. Elle s'arrête, lit l'éclat, recule. Un éclat de pierre reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La pierre de la terrasse est encore chaude. La lavande sent fort, tout près. Des tiges violettes bougent un peu. Des cigales chantent dans l'olivier. Un cerf-volant de papier attend sur la chaise. Il est bleu, avec une queue blanche. La ficelle est enroulée, un peu rêche. Je pose le chapeau sur le banc. Je remplis le verre d'eau. Tu entends les cigales, Mila ? Oui, maman. La pierre est chaude, hein ? Oui, papa. Je veux qu'il se lève. Au-dessus de la lavande. Un tout petit vent suffit. En ce moment, Mila prend le papier. Il est léger et un peu froissé.</t>
+          <t>La pierre de la terrasse tient la chaleur. Sous les paumes, elle brûle un peu. Elle est chaude, papa. Tu le sens, toi ? Oui, après la sieste. Tes yeux sont un peu lourds. Un peu, maman. Mila connaît cette terrasse. Des tiges violettes bougent près du mur. La lavande sent fort, près des pieds. Je pose le chapeau sur le banc. Je remplis le verre d'eau. Tu entends les cigales, Mila ? Oui, maman. Des cigales chantent dans l'olivier. Un cerf-volant de papier attend sur la chaise. Il est bleu, avec une queue blanche. La ficelle est rêche. Tu la tiens, Mila ? Oui, papa. Sur la pierre, un éclat de pierre brille. Il brille, maman ! Tu le vois, sur la pierre ? Oui, près de mes pieds. Je veux qu'il se lève, maintenant. Au-dessus des tiges. Un petit vent suffit. En ce moment, Mila prend le papier. Il est léger et un peu froissé. Monte ! Elle lève les bras trop vite. La ficelle claque. Le papier tombe contre les tiges. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le papier est dans les tiges. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La pierre de la terrasse est encore chaude. La lavande sent fort, tout près. Des tiges violettes bougent un peu. Des cigales chantent dans l'olivier. Un cerf-volant de papier attend sur la chaise. Il est bleu, avec une queue blanche. La ficelle est enroulée, un peu rêche. Je pose le chapeau sur le banc. Je remplis le verre d'eau. Tu entends les cigales, Mila ? Oui, maman. La pierre est chaude, hein ? Oui, papa. Je veux qu'il se lève. Au-dessus de la lavande. Un tout petit vent suffit. En ce moment, Mila prend le papier. Il est léger et un peu froissé.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La pierre de la terrasse tient la chaleur. Sous les paumes, elle brûle un peu. Elle est chaude, papa. Tu le sens, toi ? Oui, après la sieste. Tes yeux sont un peu lourds. Un peu, maman. Mila connaît cette terrasse. Des tiges violettes bougent près du mur. La lavande sent fort, près des pieds. Je pose le chapeau sur le banc. Je remplis le verre d'eau. Tu entends les cigales, Mila ? Oui, maman. Des cigales chantent dans l'olivier. Un cerf-volant de papier attend sur la chaise. Il est bleu, avec une queue blanche. La ficelle est rêche. Tu la tiens, Mila ? Oui, papa. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de pierre&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur la pierre ? Oui, près de mes pieds. Je veux qu'il se lève, maintenant. Au-dessus des tiges. Un petit vent suffit. En ce moment, Mila prend le papier. Il est léger et un peu froissé. Monte ! Elle lève les bras trop vite. La ficelle claque. Le papier tombe contre les tiges. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le papier est dans les tiges. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le sable est chaud. Un oiseau chante. Lila a envie de jouer. [pause]</t>
+          <t>La pierre de la terrasse tient la chaleur. Sous les paumes, elle brûle un peu. Elle est chaude, papa. Tu le sens, toi ? Oui, après la sieste. Tes yeux sont un peu lourds. Un peu, maman. Mila connaît cette terrasse. Des tiges violettes bougent près du mur. La lavande sent fort, près des pieds. Je pose le chapeau sur le banc. Je remplis le verre d'eau. Tu entends les cigales, Mila ? Oui, maman. Des cigales chantent dans l'olivier. Un cerf-volant de papier attend sur la chaise. Il est bleu, avec une queue blanche. La ficelle est rêche. Tu la tiens, Mila ? Oui, papa. Sur la pierre, un &lt;emphasis&gt;éclat de pierre&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur la pierre ? Oui, près de mes pieds. Je veux qu'il se lève, maintenant. Au-dessus des tiges. Un petit vent suffit. En ce moment, Mila prend le papier. Il est léger et un peu froissé. Monte ! Elle lève les bras trop vite. La ficelle claque. Le papier tombe contre les tiges. Oh. Le sourire de Mila disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je le prends ! Le papier est dans les tiges. Tu le vois, Mila ? Les épaules de Mila tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1278,28 +1278,32 @@
       <c r="AG2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pierre</t>
+        </is>
+      </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1308,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1322,27 +1326,55 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_cerf_volant_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La pierre de la terrasse est encore chaude.
-narrateur|La lavande sent fort, tout près.
-narrateur|Des tiges violettes bougent un peu.
-narrateur|Des cigales chantent dans l'olivier.
-narrateur|Un cerf-volant de papier attend sur la chaise.
-narrateur|Il est bleu, avec une queue blanche.
-narrateur|La ficelle est enroulée, un peu rêche.
+          <t>narrateur|La pierre de la terrasse tient la chaleur.
+narrateur|Sous les paumes, elle brûle un peu.
+enfant-f|Elle est chaude, papa.
+papa|Tu le sens, toi ?
+enfant-f|Oui, après la sieste.
+maman|Tes yeux sont un peu lourds.
+enfant-f|Un peu, maman.
+narrateur|Mila connaît cette terrasse.
+narrateur|Des tiges violettes bougent près du mur.
+narrateur|La lavande sent fort, près des pieds.
 maman|Je pose le chapeau sur le banc.
 papa|Je remplis le verre d'eau.
 maman|Tu entends les cigales, Mila ?
 enfant-f|Oui, maman.
-papa|La pierre est chaude, hein ?
+narrateur|Des cigales chantent dans l'olivier.
+narrateur|Un cerf-volant de papier attend sur la chaise.
+narrateur|Il est bleu, avec une queue blanche.
+enfant-f|La ficelle est rêche.
+papa|Tu la tiens, Mila ?
 enfant-f|Oui, papa.
-enfant-f|Je veux qu'il se lève.
-enfant-f|Au-dessus de la lavande.
-maman|Un tout petit vent suffit.
+narrateur|Sur la pierre, un éclat de pierre brille.
+enfant-f|Il brille, maman !
+maman|Tu le vois, sur la pierre ?
+enfant-f|Oui, près de mes pieds.
+enfant-f|Je veux qu'il se lève, maintenant.
+enfant-f|Au-dessus des tiges.
+maman|Un petit vent suffit.
 narrateur|En ce moment, Mila prend le papier.
-narrateur|Il est léger et un peu froissé.</t>
+narrateur|Il est léger et un peu froissé.
+enfant-f|Monte !
+narrateur|Elle lève les bras trop vite.
+narrateur|La ficelle claque.
+narrateur|Le papier tombe contre les tiges.
+enfant-f|Oh.
+narrateur|Le sourire de Mila disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je le prends !
+maman|Le papier est dans les tiges.
+papa|Tu le vois, Mila ?
+narrateur|Les épaules de Mila tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1374,17 +1406,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Aniss est sur la marche. Ses pieds restent à l'ombre. Mila tient la ficelle. Tu viens ? Je regarde. Mila accepte. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Mila lève le papier. Le vent le fait trembler. Aniss reste sur la marche. Il regarde la queue blanche. Plus tard ? Plus tard. D'accord. Tu as accepté, Mila ? Oui, papa. Regarder, c'est une réponse. Une abeille passe sur la lavande. Elle fait un petit bruit. Tu l'entends, Mila ? Oui. On attend qu'elle parte. Mila tient le papier bas. L'abeille s'en va. Tu veux la ficelle ? Non. D'accord. Plusieurs réponses sont possibles. Le cerf-volant tremble encore. Aniss avance un pied. Puis il le retire.</t>
+          <t>Aniss est sur la marche. Ses pieds restent à l'ombre. Tu viens ? Aniss ne dit rien. Mila tient la ficelle trop près. Prends-la, maintenant ! Elle pousse la ficelle vers sa main. Aniss retire les doigts. Je regarde. Oh. Le papier tremble, trop bas. Le papier reste sous les tiges. Tu l'as vu, le papier ? Il ne se lève pas. Aniss est sur la marche. Plus tard ? Plus tard. Mila avance d'un pas. Aniss recule le pied. Tu veux la ficelle ? Non. La queue blanche traîne. Une abeille passe sur les tiges. Tu l'entends, Mila ? Oui. On attend qu'elle parte. Mila tient le papier bas. L'abeille s'en va. Les épaules restent basses.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Aniss est sur la marche. Ses pieds restent à l'ombre. Mila tient la ficelle. Tu viens ? Je regarde. Mila accepte. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Mila lève le papier. Le vent le fait trembler. Aniss reste sur la marche. Il regarde la queue blanche. Plus tard ? Plus tard. D'accord. Tu as accepté, Mila ? Oui, papa. Regarder, c'est une réponse. Une abeille passe sur la lavande. Elle fait un petit bruit. Tu l'entends, Mila ? Oui. On attend qu'elle parte. Mila tient le papier bas. L'abeille s'en va. Tu veux la ficelle ? Non. D'accord. Plusieurs réponses sont possibles. Le cerf-volant tremble encore. Aniss avance un pied. Puis il le retire.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Aniss est sur la marche. Ses pieds restent à l'ombre. Tu viens ? Aniss ne dit rien. Mila tient la ficelle trop près. Prends-la, maintenant ! Elle pousse la ficelle vers sa main. Aniss retire les doigts. &lt;emphasis level="moderate"&gt;Je regarde&lt;/emphasis&gt;. Oh. Le papier tremble, trop bas. Le papier reste sous les tiges. Tu l'as vu, le papier ? Il ne se lève pas. Aniss est sur la marche. Plus tard ? Plus tard. Mila avance d'un pas. Aniss recule le pied. Tu veux la ficelle ? Non. La queue blanche traîne. Une abeille passe sur les tiges. Tu l'entends, Mila ? Oui. On attend qu'elle parte. Mila tient le papier bas. L'abeille s'en va. Les épaules restent basses.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Lila est au parc avec maman. Kenzo est près du bac. Lila va &lt;emphasis&gt;proposer&lt;/emphasis&gt; le seau. Elle dit : tu viens ? Kenzo dit : je regarde. Lila accepte. Maman dit : on peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Lila creuse. Kenzo reste au bord. Lila propose encore, tout doux : plus tard ? Kenzo dit : plus tard. Lila dit : d'accord. Elle accepte plusieurs réponses. [pause]</t>
+          <t>&lt;low-pitch&gt;Aniss est sur la marche. Ses pieds restent à l'ombre. Tu viens ? Aniss ne dit rien. Mila tient la ficelle trop près. Prends-la, maintenant ! Elle pousse la ficelle vers sa main. Aniss retire les doigts. &lt;emphasis&gt;Je regarde&lt;/emphasis&gt;. Oh. Le papier tremble, trop bas. Le papier reste sous les tiges. Tu l'as vu, le papier ? Il ne se lève pas. Aniss est sur la marche. Plus tard ? Plus tard. Mila avance d'un pas. Aniss recule le pied. Tu veux la ficelle ? Non. La queue blanche traîne. Une abeille passe sur les tiges. Tu l'entends, Mila ? Oui. On attend qu'elle parte. Mila tient le papier bas. L'abeille s'en va. Les épaules restent basses.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1431,7 +1463,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1439,22 +1471,26 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE3" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF3" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1465,30 +1501,30 @@
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>Je regarde</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1497,60 +1533,56 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS3" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT3" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU3" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV3" s="2" t="inlineStr"/>
+      <c r="AV3" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis retenue; intensite=2; destinataire=enfant; sous_texte=aniss_regarde_ne_prend_pas_la_ficelle; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Aniss est sur la marche.
 narrateur|Ses pieds restent à l'ombre.
-narrateur|Mila tient la ficelle.
 enfant-f|Tu viens ?
+narrateur|Aniss ne dit rien.
+narrateur|Mila tient la ficelle trop près.
+enfant-f|Prends-la, maintenant !
+narrateur|Elle pousse la ficelle vers sa main.
+narrateur|Aniss retire les doigts.
 copain|Je regarde.
-narrateur|Mila accepte.
-maman|On peut proposer.
-maman|On peut accepter plusieurs réponses.
-papa|Oui.
-papa|Non.
-papa|Regarder.
-papa|Plus tard.
-enfant-f|D'accord.
-narrateur|Mila lève le papier.
-narrateur|Le vent le fait trembler.
-narrateur|Aniss reste sur la marche.
-narrateur|Il regarde la queue blanche.
+enfant-f|Oh.
+narrateur|Le papier tremble, trop bas.
+narrateur|Le papier reste sous les tiges.
+papa|Tu l'as vu, le papier ?
+enfant-f|Il ne se lève pas.
+maman|Aniss est sur la marche.
 enfant-f|Plus tard ?
 copain|Plus tard.
-enfant-f|D'accord.
-papa|Tu as accepté, Mila ?
-enfant-f|Oui, papa.
-maman|Regarder, c'est une réponse.
-narrateur|Une abeille passe sur la lavande.
-narrateur|Elle fait un petit bruit.
+narrateur|Mila avance d'un pas.
+narrateur|Aniss recule le pied.
+enfant-f|Tu veux la ficelle ?
+copain|Non.
+narrateur|La queue blanche traîne.
+narrateur|Une abeille passe sur les tiges.
 maman|Tu l'entends, Mila ?
 enfant-f|Oui.
 papa|On attend qu'elle parte.
 narrateur|Mila tient le papier bas.
 narrateur|L'abeille s'en va.
-enfant-f|Tu veux la ficelle ?
-copain|Non.
-enfant-f|D'accord.
-papa|Plusieurs réponses sont possibles.
-narrateur|Le cerf-volant tremble encore.
-narrateur|Aniss avance un pied.
-narrateur|Puis il le retire.</t>
+narrateur|Les épaules restent basses.</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
@@ -1587,12 +1619,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila invite Aniss. Que fait-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila &lt;emphasis level="moderate"&gt;invite&lt;/emphasis&gt; Aniss. Que fait-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Lila invite Kenzo. Que fait-elle si Kenzo dit non ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila &lt;emphasis&gt;invite&lt;/emphasis&gt; Aniss. Que fait-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1655,7 +1687,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1666,7 +1698,7 @@
         <v>0.86</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1681,34 +1713,38 @@
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>invite</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1723,17 +1759,17 @@
         <v>0.86</v>
       </c>
       <c r="AS4" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT4" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_invite_et_prend_la_reponse_d_aniss; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
@@ -1766,17 +1802,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Mila a su proposer. Elle a su accepter plusieurs réponses. Aniss a dit regarder, puis plus tard. Oui. Tout ça va. J'ai dit d'accord. Bravo. Tu as tenu la ficelle. Le papier se lève un peu. L'ombre passe sur la lavande. Tu vois l'ombre, Aniss ? Je regarde. C'est une réponse. Mila recule d'un pas. La queue blanche danse. Une tige de lavande se plie. Le vent est juste assez.</t>
+          <t>Mila avance trop vite vers Aniss. Tu viens, maintenant ! Sa voix se mélange au vent. Oh. Aniss reste sur la marche. Mila refuse de foncer. Elle referme la main. Elle regarde la pierre, un instant. Tu veux venir près de la pierre ? Papa s'accroupit à la même hauteur. Mila pose un pied sur la pierre chaude. Tu viens ? Elle attend. Aniss ne dit rien. D'accord. Je regarde. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Sur la pierre, un éclat de pierre tient. Il est là. Mila lève le papier, sans tirer. Un petit vent prend la queue. Je vois. Il tremble un peu. Il se lève.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Mila a su proposer. Elle a su accepter plusieurs réponses. Aniss a dit regarder, puis plus tard. Oui. Tout ça va. J'ai dit d'accord. Bravo. Tu as tenu la ficelle. Le papier se lève un peu. L'ombre passe sur la lavande. Tu vois l'ombre, Aniss ? Je regarde. C'est une réponse. Mila recule d'un pas. La queue blanche danse. Une tige de lavande se plie. Le vent est juste assez.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila avance trop vite vers Aniss. Tu viens, maintenant ! Sa voix se mélange au vent. Oh. Aniss reste sur la marche. Mila refuse de foncer. Elle referme la main. Elle regarde la pierre, un instant. Tu veux venir près de la pierre ? Papa s'accroupit à la même hauteur. Mila pose un pied sur la pierre chaude. Tu viens ? Elle attend. Aniss ne dit rien. &lt;emphasis level="moderate"&gt;D'accord&lt;/emphasis&gt;. Je regarde. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Sur la pierre, un éclat de pierre tient. Il est là. Mila lève le papier, sans tirer. Un petit vent prend la queue. Je vois. Il tremble un peu. Il se lève.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Lila a su &lt;emphasis&gt;proposer&lt;/emphasis&gt;. Elle a su accepter plusieurs réponses. [pause]</t>
+          <t>Mila avance trop vite vers Aniss. Tu viens, maintenant ! Sa voix se mélange au vent. Oh. Aniss reste sur la marche. Mila refuse de foncer. Elle referme la main. Elle regarde la pierre, un instant. Tu veux venir près de la pierre ? Papa s'accroupit à la même hauteur. Mila pose un pied sur la pierre chaude. Tu viens ? Elle attend. Aniss ne dit rien. &lt;emphasis&gt;D'accord&lt;/emphasis&gt;. Je regarde. Merci, Mila. Papa a entendu toute la phrase. Le ventre de Mila se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, maman. Sur la pierre, un éclat de pierre tient. Il est là. Mila lève le papier, sans tirer. Un petit vent prend la queue. Je vois. Il tremble un peu. Il se lève. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,7 +1859,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1831,10 +1867,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,30 +1893,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>D'accord</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1889,10 +1925,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1905,28 +1941,40 @@
       </c>
       <c r="AV5" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=d_accord_laisse_aniss_regarder; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Mila a su proposer.
-narrateur|Elle a su accepter plusieurs réponses.
-papa|Aniss a dit regarder, puis plus tard.
-maman|Oui.
-maman|Tout ça va.
-enfant-f|J'ai dit d'accord.
-papa|Bravo.
-papa|Tu as tenu la ficelle.
-narrateur|Le papier se lève un peu.
-narrateur|L'ombre passe sur la lavande.
-enfant-f|Tu vois l'ombre, Aniss ?
+          <t>narrateur|Mila avance trop vite vers Aniss.
+enfant-f|Tu viens, maintenant !
+narrateur|Sa voix se mélange au vent.
+enfant-f|Oh.
+narrateur|Aniss reste sur la marche.
+narrateur|Mila refuse de foncer.
+narrateur|Elle referme la main.
+narrateur|Elle regarde la pierre, un instant.
+papa|Tu veux venir près de la pierre ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Mila pose un pied sur la pierre chaude.
+enfant-f|Tu viens ?
+narrateur|Elle attend.
+narrateur|Aniss ne dit rien.
+enfant-f|D'accord.
 copain|Je regarde.
-maman|C'est une réponse.
-narrateur|Mila recule d'un pas.
-narrateur|La queue blanche danse.
-narrateur|Une tige de lavande se plie.
-papa|Le vent est juste assez.</t>
+papa|Merci, Mila.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Mila se desserre.
+narrateur|Les épaules se relèvent un peu.
+maman|Tu as les mains au chaud ?
+enfant-f|Un peu, maman.
+narrateur|Sur la pierre, un éclat de pierre tient.
+enfant-f|Il est là.
+narrateur|Mila lève le papier, sans tirer.
+narrateur|Un petit vent prend la queue.
+copain|Je vois.
+maman|Il tremble un peu.
+enfant-f|Il se lève.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1958,17 +2006,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On repose le papier ? Encore un peu. L'ombre glisse sur deux tiges. Aniss suit des yeux. Tu as fini de jouer, Mila ? Oui, papa. Mila pose le cerf-volant. Il retrouve la chaise. Aniss secoue un pied. Un peu de poussière tombe. Merci, Aniss. Tu as regardé. La lavande sent encore. L'ombre était jolie. Oui.</t>
+          <t>Mila tire la ficelle trop vite. Au-dessus des tiges, d'un coup ! Le papier plonge dans les tiges. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila observe la pierre, écoute les cigales. Sur la pierre, un éclat de pierre luit. Là, près de mes pieds. Mila recule d'un pas. Elle tient la ficelle des deux mains. Il est léger, papa. Tu le portes vers le vent ? Oui, papa. On avance ? Oui, maman. Un petit vent arrive. Le papier se lève un peu. L'ombre passe sur les tiges. Tu vois l'ombre, Aniss ? Je regarde. Aniss avance un pied. Puis il le retire. D'accord. On reste là. La queue blanche danse. Une tige violette se plie. Le vent est juste assez.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On repose le papier ? Encore un peu. L'ombre glisse sur deux tiges. Aniss suit des yeux. Tu as fini de jouer, Mila ? Oui, papa. Mila pose le cerf-volant. Il retrouve la chaise. Aniss secoue un pied. Un peu de poussière tombe. Merci, Aniss. Tu as regardé. La lavande sent encore. L'ombre était jolie. Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Mila tire la ficelle trop vite. Au-dessus des tiges, d'un coup ! Le papier plonge dans les tiges. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila observe la pierre, écoute les cigales. Sur la pierre, un &lt;emphasis level="moderate"&gt;éclat de pierre&lt;/emphasis&gt; luit. Là, près de mes pieds. Mila recule d'un pas. Elle tient la ficelle des deux mains. Il est léger, papa. Tu le portes vers le vent ? Oui, papa. On avance ? Oui, maman. Un petit vent arrive. Le papier se lève un peu. L'ombre passe sur les tiges. Tu vois l'ombre, Aniss ? Je regarde. Aniss avance un pied. Puis il le retire. D'accord. On reste là. La queue blanche danse. Une tige violette se plie. Le vent est juste assez.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Maman range le seau. Lila donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Mila tire la ficelle trop vite. Au-dessus des tiges, d'un coup ! Le papier plonge dans les tiges. Oh. Mila avance les mains. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Mila observe la pierre, écoute les cigales. Sur la pierre, un &lt;emphasis&gt;éclat de pierre&lt;/emphasis&gt; luit. Là, près de mes pieds. Mila recule d'un pas. Elle tient la ficelle des deux mains. Il est léger, papa. Tu le portes vers le vent ? Oui, papa. On avance ? Oui, maman. Un petit vent arrive. Le papier se lève un peu. L'ombre passe sur les tiges. Tu vois l'ombre, Aniss ? Je regarde. Aniss avance un pied. Puis il le retire. D'accord. On reste là. La queue blanche danse. Une tige violette se plie. Le vent est juste assez. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2015,7 +2063,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2023,10 +2071,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2049,30 +2097,30 @@
       </c>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de pierre</t>
         </is>
       </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2081,10 +2129,10 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS6" s="2" t="n">
         <v>100</v>
@@ -2095,24 +2143,48 @@
       <c r="AU6" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat_de_pierre; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>maman|On repose le papier ?
-enfant-f|Encore un peu.
-narrateur|L'ombre glisse sur deux tiges.
-narrateur|Aniss suit des yeux.
-papa|Tu as fini de jouer, Mila ?
+          <t>narrateur|Mila tire la ficelle trop vite.
+enfant-f|Au-dessus des tiges, d'un coup !
+narrateur|Le papier plonge dans les tiges.
+enfant-f|Oh.
+narrateur|Mila avance les mains.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Mila observe la pierre, écoute les cigales.
+narrateur|Sur la pierre, un éclat de pierre luit.
+enfant-f|Là, près de mes pieds.
+narrateur|Mila recule d'un pas.
+narrateur|Elle tient la ficelle des deux mains.
+enfant-f|Il est léger, papa.
+papa|Tu le portes vers le vent ?
 enfant-f|Oui, papa.
-narrateur|Mila pose le cerf-volant.
-narrateur|Il retrouve la chaise.
-narrateur|Aniss secoue un pied.
-narrateur|Un peu de poussière tombe.
-maman|Merci, Aniss.
-maman|Tu as regardé.
-papa|La lavande sent encore.
-enfant-f|L'ombre était jolie.
-papa|Oui.</t>
+maman|On avance ?
+enfant-f|Oui, maman.
+narrateur|Un petit vent arrive.
+narrateur|Le papier se lève un peu.
+narrateur|L'ombre passe sur les tiges.
+enfant-f|Tu vois l'ombre, Aniss ?
+copain|Je regarde.
+narrateur|Aniss avance un pied.
+narrateur|Puis il le retire.
+enfant-f|D'accord.
+maman|On reste là.
+narrateur|La queue blanche danse.
+narrateur|Une tige violette se plie.
+papa|Le vent est juste assez.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>vent,papier</t>
         </is>
       </c>
     </row>
@@ -2139,17 +2211,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Le cerf-volant bleu dort sur la chaise. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. Les cigales chantent encore.</t>
+          <t>Le papier brillait, papa. Tu le vois, comme sur la chaise ? Oui, un peu froissé. Mila pose le cerf-volant. Il retrouve la chaise. On le garde près de nous ? Oui, maman. La lavande sentait fort. Les tiges sont derrière nous. Aniss secoue un pied. Un peu de poussière tombe. On rentre ? Oui. Les joues de Mila se réchauffent. La pierre reste chaude sous la main. Elle est chaude. Comme tout à l'heure ? Oui, maman. La lumière est pâle, toi ? Oui, papa. Un éclat de pierre reste pâle.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Le cerf-volant bleu dort sur la chaise. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. Les cigales chantent encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le papier brillait, papa. Tu le vois, comme sur la chaise ? Oui, un peu froissé. Mila pose le cerf-volant. Il retrouve la chaise. On le garde près de nous ? Oui, maman. La lavande sentait fort. Les tiges sont derrière nous. Aniss secoue un pied. Un peu de poussière tombe. On rentre ? Oui. Les joues de Mila se réchauffent. La pierre reste chaude sous la main. Elle est chaude. Comme tout à l'heure ? Oui, maman. La lumière est pâle, toi ? Oui, papa. Un &lt;emphasis level="moderate"&gt;éclat de pierre&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le papier brillait, papa. Tu le vois, comme sur la chaise ? Oui, un peu froissé. Mila pose le cerf-volant. Il retrouve la chaise. On le garde près de nous ? Oui, maman. La lavande sentait fort. Les tiges sont derrière nous. Aniss secoue un pied. Un peu de poussière tombe. On rentre ? Oui. Les joues de Mila se réchauffent. La pierre reste chaude sous la main. Elle est chaude. Comme tout à l'heure ? Oui, maman. La lumière est pâle, toi ? Oui, papa. Un &lt;emphasis&gt;éclat de pierre&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -2196,18 +2268,18 @@
         </is>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
@@ -2216,12 +2288,12 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF7" s="2" t="inlineStr">
@@ -2230,17 +2302,21 @@
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH7" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH7" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pierre</t>
+        </is>
+      </c>
       <c r="AI7" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL7" s="2" t="inlineStr">
         <is>
@@ -2249,11 +2325,11 @@
       </c>
       <c r="AM7" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO7" s="2" t="inlineStr"/>
       <c r="AP7" s="2" t="inlineStr">
@@ -2262,29 +2338,53 @@
         </is>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT7" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV7" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV7" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_pierre_reste_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|Le cerf-volant bleu dort sur la chaise.
-enfant-f|J'ai proposé.
-enfant-f|J'ai accepté.
-maman|Plusieurs réponses sont possibles.
-papa|Oui.
-narrateur|Les cigales chantent encore.</t>
+          <t>enfant-f|Le papier brillait, papa.
+papa|Tu le vois, comme sur la chaise ?
+enfant-f|Oui, un peu froissé.
+narrateur|Mila pose le cerf-volant.
+narrateur|Il retrouve la chaise.
+maman|On le garde près de nous ?
+enfant-f|Oui, maman.
+enfant-f|La lavande sentait fort.
+maman|Les tiges sont derrière nous.
+narrateur|Aniss secoue un pied.
+narrateur|Un peu de poussière tombe.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Mila se réchauffent.
+narrateur|La pierre reste chaude sous la main.
+enfant-f|Elle est chaude.
+maman|Comme tout à l'heure ?
+enfant-f|Oui, maman.
+papa|La lumière est pâle, toi ?
+enfant-f|Oui, papa.
+narrateur|Un éclat de pierre reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>terrasse</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2383,6 +2483,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>